<commit_message>
feat: add App_1_32 human fighter appearance prefab and catalogs
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Mode2/Excel/制造_躯体外观配置表_Manufacture_BodyAppearanceConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Mode2/Excel/制造_躯体外观配置表_Manufacture_BodyAppearanceConfig.xlsx
@@ -1127,7 +1127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="9" customWidth="1" style="6" min="2" max="2"/>
@@ -2253,7 +2253,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>App_1_33</t>
+          <t>App_1_32</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2266,12 +2266,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>影刃</t>
+          <t>格斗师</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>瞬移后排</t>
+          <t>专供精英敌人</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -2293,7 +2293,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>App_2_02</t>
+          <t>App_1_33</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2301,17 +2301,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Race_Elf</t>
+          <t>Race_Human</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>近卫</t>
+          <t>影刃</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>高防御战士</t>
+          <t>瞬移后排</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -2333,7 +2333,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>App_2_03</t>
+          <t>App_2_02</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2346,12 +2346,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>狂战士</t>
+          <t>近卫</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>高伤害</t>
+          <t>高防御战士</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -2373,7 +2373,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>App_2_12</t>
+          <t>App_2_03</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -2386,12 +2386,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>炸弹师</t>
+          <t>狂战士</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>范围爆炸</t>
+          <t>高伤害</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -2413,7 +2413,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>App_2_13</t>
+          <t>App_2_12</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -2426,12 +2426,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>长弓手</t>
+          <t>炸弹师</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>直线贯穿</t>
+          <t>范围爆炸</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -2453,7 +2453,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>App_2_22</t>
+          <t>App_2_13</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -2466,12 +2466,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>冰法</t>
+          <t>长弓手</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>减速冰冻</t>
+          <t>直线贯穿</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -2493,7 +2493,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>App_2_23</t>
+          <t>App_2_22</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -2506,12 +2506,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>火法</t>
+          <t>冰法</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>范围持续伤害</t>
+          <t>减速冰冻</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -2533,7 +2533,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>App_2_32</t>
+          <t>App_2_23</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2546,12 +2546,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>格斗师</t>
+          <t>火法</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>专供精英敌人</t>
+          <t>范围持续伤害</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -2573,7 +2573,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>App_2_33</t>
+          <t>App_2_32</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -2586,12 +2586,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>影刃</t>
+          <t>格斗师</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>瞬移后排</t>
+          <t>专供精英敌人</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -2613,7 +2613,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>App_3_02</t>
+          <t>App_2_33</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2621,17 +2621,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Race_Orc</t>
+          <t>Race_Elf</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>近卫</t>
+          <t>影刃</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>高防御战士</t>
+          <t>瞬移后排</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -2653,7 +2653,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>App_3_03</t>
+          <t>App_3_02</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -2666,12 +2666,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>狂战士</t>
+          <t>近卫</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>高伤害</t>
+          <t>高防御战士</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2693,7 +2693,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>App_3_12</t>
+          <t>App_3_03</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2706,12 +2706,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>炸弹师</t>
+          <t>狂战士</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>范围爆炸</t>
+          <t>高伤害</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -2733,7 +2733,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>App_3_13</t>
+          <t>App_3_12</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2746,12 +2746,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>长弓手</t>
+          <t>炸弹师</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>直线贯穿</t>
+          <t>范围爆炸</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -2773,7 +2773,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>App_3_22</t>
+          <t>App_3_13</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2786,12 +2786,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>冰法</t>
+          <t>长弓手</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>减速冰冻</t>
+          <t>直线贯穿</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -2813,7 +2813,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>App_3_23</t>
+          <t>App_3_22</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -2826,12 +2826,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>火法</t>
+          <t>冰法</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>范围持续伤害</t>
+          <t>减速冰冻</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -2853,7 +2853,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>App_3_32</t>
+          <t>App_3_23</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2866,12 +2866,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>格斗师</t>
+          <t>火法</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>专供精英敌人</t>
+          <t>范围持续伤害</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -2893,40 +2893,80 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>App_3_32</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>3</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Race_Orc</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>格斗师</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>专供精英敌人</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>App_3_33</t>
         </is>
       </c>
-      <c r="B44" t="n">
-        <v>3</v>
-      </c>
-      <c r="C44" t="inlineStr">
+      <c r="B45" t="n">
+        <v>3</v>
+      </c>
+      <c r="C45" t="inlineStr">
         <is>
           <t>Race_Orc</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>影刃</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>瞬移后排</t>
         </is>
       </c>
-      <c r="F44" t="n">
-        <v>1</v>
-      </c>
-      <c r="G44" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="H44" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="I44" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="J44" t="n">
+      <c r="F45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J45" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>